<commit_message>
Mover archivos de análisis a 02_Planning junto con fuentes
Los Excel generados por los scripts de análisis (Analisis_Cronogramas,
Analisis_Comparativo, Hitos_Generales, Gantt_Cadena_Critica) se
reubican en 02_Planning/ junto al Gantt ABB y el XER de Primavera.
Scripts actualizados para guardar en PLANNING_DIR por defecto.

https://claude.ai/code/session_017wF27KL2NtMGeTJBXCBM3L
</commit_message>
<xml_diff>
--- a/ABB_Proyecto/01_Ofertas/Ofertas.xlsx
+++ b/ABB_Proyecto/01_Ofertas/Ofertas.xlsx
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>46165</v>
+        <v>46167</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>46165</v>
+        <v>46167</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>

</xml_diff>